<commit_message>
Update User_Data_Template and Add User Page to not require date of birth and place of birth for admin roles
</commit_message>
<xml_diff>
--- a/public/documents/user_templates/User_Data_Template.xlsx
+++ b/public/documents/user_templates/User_Data_Template.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Deonn Lansangan\Downloads\v1.2.3 hauoieidmo-main\public\documents\user_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{72778E1A-1524-40A9-9EAA-0E5BBE6CD20A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F5DB3CA-ABF1-4588-9075-494DD96377DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180" firstSheet="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Login_Info" sheetId="7" r:id="rId1"/>
-    <sheet name="Personal_Info" sheetId="1" r:id="rId2"/>
-    <sheet name="Contact_Info" sheetId="2" r:id="rId3"/>
-    <sheet name="Prov_Contact_Info" sheetId="3" r:id="rId4"/>
-    <sheet name="Em_Contact_Info" sheetId="4" r:id="rId5"/>
-    <sheet name="Acc_Details" sheetId="5" r:id="rId6"/>
-    <sheet name="Hiring_Info" sheetId="6" r:id="rId7"/>
+    <sheet name="Guide" sheetId="8" r:id="rId1"/>
+    <sheet name="Login_Info" sheetId="7" r:id="rId2"/>
+    <sheet name="Personal_Info" sheetId="1" r:id="rId3"/>
+    <sheet name="Contact_Info" sheetId="2" r:id="rId4"/>
+    <sheet name="Prov_Contact_Info" sheetId="3" r:id="rId5"/>
+    <sheet name="Em_Contact_Info" sheetId="4" r:id="rId6"/>
+    <sheet name="Acc_Details" sheetId="5" r:id="rId7"/>
+    <sheet name="Hiring_Info" sheetId="6" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -42,7 +43,181 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="88">
+  <si>
+    <t>Guidelines</t>
+  </si>
+  <si>
+    <t>Fill in the required fields based on the role of the user</t>
+  </si>
+  <si>
+    <t>Sample data is provided in the sheets for reference</t>
+  </si>
+  <si>
+    <t>ADMIN ROLES: SuperAdmin, HR Admin, Dean, IDC Admin, ISO Document Handler</t>
+  </si>
+  <si>
+    <t>EMPLOYEE ROLE: Any role NOT listed as an Admin role</t>
+  </si>
+  <si>
+    <t>DATE FORMAT: Use MM/DD/YYYY (e.g., 02/24/2003)</t>
+  </si>
+  <si>
+    <t>CONDITIONAL REQUIREMENT: Non Tenured field becomes REQUIRED when Tenure = "Non-tenured"</t>
+  </si>
+  <si>
+    <t>VALIDATION RULES</t>
+  </si>
+  <si>
+    <t>Sheet Name</t>
+  </si>
+  <si>
+    <t>Field Name</t>
+  </si>
+  <si>
+    <t>Admin Roles</t>
+  </si>
+  <si>
+    <t>Employee Role</t>
+  </si>
+  <si>
+    <t>Login_Info</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>✓ REQUIRED</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>Personal_Info</t>
+  </si>
+  <si>
+    <t>Employee ID</t>
+  </si>
+  <si>
+    <t>First Name</t>
+  </si>
+  <si>
+    <t>Middle Name</t>
+  </si>
+  <si>
+    <t>OPTIONAL</t>
+  </si>
+  <si>
+    <t>Last Name</t>
+  </si>
+  <si>
+    <t>Department</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Maiden Name</t>
+  </si>
+  <si>
+    <t>Date of Birth</t>
+  </si>
+  <si>
+    <t>Place of Birth</t>
+  </si>
+  <si>
+    <t>Civil Status</t>
+  </si>
+  <si>
+    <t>Religion</t>
+  </si>
+  <si>
+    <t>Blood Type</t>
+  </si>
+  <si>
+    <t>Contact_Info</t>
+  </si>
+  <si>
+    <t>House Number</t>
+  </si>
+  <si>
+    <t>Street</t>
+  </si>
+  <si>
+    <t>Barangay</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Province</t>
+  </si>
+  <si>
+    <t>Postal Code</t>
+  </si>
+  <si>
+    <t>Home Phone</t>
+  </si>
+  <si>
+    <t>Mobile Phone</t>
+  </si>
+  <si>
+    <t>Email Address 1</t>
+  </si>
+  <si>
+    <t>Email Address 2</t>
+  </si>
+  <si>
+    <t>Prov_Contact_Info</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>Em_Contact_Info</t>
+  </si>
+  <si>
+    <t>Relationship</t>
+  </si>
+  <si>
+    <t>Acc_Details</t>
+  </si>
+  <si>
+    <t>SSS Number</t>
+  </si>
+  <si>
+    <t>TIN</t>
+  </si>
+  <si>
+    <t>Pag-IBIG Number</t>
+  </si>
+  <si>
+    <t>PhilHealth Number</t>
+  </si>
+  <si>
+    <t>Hiring_Info</t>
+  </si>
+  <si>
+    <t>Date Hired</t>
+  </si>
+  <si>
+    <t>Position</t>
+  </si>
+  <si>
+    <t>Nature</t>
+  </si>
+  <si>
+    <t>Tenure</t>
+  </si>
+  <si>
+    <t>Non Tenured</t>
+  </si>
+  <si>
+    <t>Required License</t>
+  </si>
   <si>
     <r>
       <rPr>
@@ -89,15 +264,6 @@
     <t>system from reading the data correctly.</t>
   </si>
   <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Role</t>
-  </si>
-  <si>
-    <t>Password</t>
-  </si>
-  <si>
     <t>sample@gmail.com</t>
   </si>
   <si>
@@ -107,45 +273,15 @@
     <t>password</t>
   </si>
   <si>
+    <t>sample2@gmail.com</t>
+  </si>
+  <si>
+    <t>SuperAdmin</t>
+  </si>
+  <si>
     <t>Personal Information</t>
   </si>
   <si>
-    <t>Employee ID</t>
-  </si>
-  <si>
-    <t>First Name</t>
-  </si>
-  <si>
-    <t>Middle Name</t>
-  </si>
-  <si>
-    <t>Last Name</t>
-  </si>
-  <si>
-    <t>Department</t>
-  </si>
-  <si>
-    <t>Gender</t>
-  </si>
-  <si>
-    <t>Maiden Name</t>
-  </si>
-  <si>
-    <t>Date of Birth</t>
-  </si>
-  <si>
-    <t>Place of Birth</t>
-  </si>
-  <si>
-    <t>Civil Status</t>
-  </si>
-  <si>
-    <t>Religion</t>
-  </si>
-  <si>
-    <t>Blood Type</t>
-  </si>
-  <si>
     <t>Records Systems and Services</t>
   </si>
   <si>
@@ -161,85 +297,22 @@
     <t>Contact Information</t>
   </si>
   <si>
-    <t>House Number</t>
-  </si>
-  <si>
-    <t>Street</t>
-  </si>
-  <si>
-    <t>Barangay</t>
-  </si>
-  <si>
-    <t>City</t>
-  </si>
-  <si>
-    <t>Province</t>
-  </si>
-  <si>
-    <t>Postal Code</t>
-  </si>
-  <si>
-    <t>Home Phone</t>
-  </si>
-  <si>
-    <t>Mobile Phone</t>
-  </si>
-  <si>
-    <t>Email Address 1</t>
-  </si>
-  <si>
-    <t>Email Address 2</t>
-  </si>
-  <si>
-    <t>sample2@gmail.com</t>
-  </si>
-  <si>
     <t>Provincial Contact</t>
   </si>
   <si>
-    <t>Phone</t>
-  </si>
-  <si>
     <t>Emergency Information</t>
   </si>
   <si>
-    <t>Relationship</t>
-  </si>
-  <si>
     <t>Accounting Details</t>
   </si>
   <si>
-    <t>SSS Number</t>
-  </si>
-  <si>
     <t>Tax Identification Number</t>
   </si>
   <si>
     <t>Pag IBIG Number</t>
   </si>
   <si>
-    <t>PhilHealth Number</t>
-  </si>
-  <si>
     <t>Hiring Information</t>
-  </si>
-  <si>
-    <t>Date Hired</t>
-  </si>
-  <si>
-    <t>Position</t>
-  </si>
-  <si>
-    <t>Nature</t>
-  </si>
-  <si>
-    <t>Tenure</t>
-  </si>
-  <si>
-    <t>Non Tenured</t>
-  </si>
-  <si>
-    <t>Required License</t>
   </si>
   <si>
     <t>Faculty</t>
@@ -258,7 +331,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -327,8 +400,55 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -353,12 +473,141 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE699"/>
+        <bgColor rgb="FFFFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF751E1B"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -367,7 +616,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -398,18 +647,71 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -690,8 +992,780 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF0F9748-D1A2-4B51-9B51-41F1F2B97E8D}">
+  <dimension ref="A1:D71"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" customWidth="1"/>
+    <col min="4" max="4" width="23.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="35.1" customHeight="1">
+      <c r="A1" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="30"/>
+    </row>
+    <row r="2" spans="1:4" ht="15" customHeight="1">
+      <c r="A2" s="35" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="37"/>
+    </row>
+    <row r="3" spans="1:4" ht="16.5" customHeight="1">
+      <c r="A3" s="38" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="40"/>
+    </row>
+    <row r="4" spans="1:4" ht="15" customHeight="1">
+      <c r="A4" s="34"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="33"/>
+    </row>
+    <row r="5" spans="1:4" ht="15" customHeight="1">
+      <c r="A5" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="19"/>
+    </row>
+    <row r="6" spans="1:4" ht="15" customHeight="1">
+      <c r="A6" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="19"/>
+    </row>
+    <row r="7" spans="1:4" ht="15" customHeight="1">
+      <c r="A7" s="31"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="33"/>
+    </row>
+    <row r="8" spans="1:4" ht="15" customHeight="1">
+      <c r="A8" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="19"/>
+    </row>
+    <row r="9" spans="1:4" ht="15" customHeight="1">
+      <c r="A9" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="19"/>
+    </row>
+    <row r="10" spans="1:4" ht="16.5" customHeight="1"/>
+    <row r="11" spans="1:4" ht="42.75" customHeight="1">
+      <c r="A11" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+    </row>
+    <row r="12" spans="1:4" ht="15" customHeight="1">
+      <c r="A12" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="22" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="21" customHeight="1">
+      <c r="A13" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A14" s="26"/>
+      <c r="B14" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="18" customHeight="1">
+      <c r="A15" s="26"/>
+      <c r="B15" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="19.5" customHeight="1">
+      <c r="A16" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="18.75" customHeight="1">
+      <c r="A17" s="26"/>
+      <c r="B17" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="26"/>
+      <c r="B18" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D18" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="16.5">
+      <c r="A19" s="26"/>
+      <c r="B19" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="16.5">
+      <c r="A20" s="26"/>
+      <c r="B20" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="26"/>
+      <c r="B21" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D21" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="26"/>
+      <c r="B22" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D22" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="16.5">
+      <c r="A23" s="26"/>
+      <c r="B23" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="16.5">
+      <c r="A24" s="26"/>
+      <c r="B24" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D24" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="26"/>
+      <c r="B25" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D25" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="26"/>
+      <c r="B26" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D26" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="26"/>
+      <c r="B27" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D27" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="16.5">
+      <c r="A28" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D28" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="16.5">
+      <c r="A29" s="26"/>
+      <c r="B29" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C29" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D29" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="16.5">
+      <c r="A30" s="26"/>
+      <c r="B30" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="C30" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D30" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="16.5">
+      <c r="A31" s="26"/>
+      <c r="B31" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C31" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D31" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="16.5">
+      <c r="A32" s="26"/>
+      <c r="B32" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="C32" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D32" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="16.5">
+      <c r="A33" s="26"/>
+      <c r="B33" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="C33" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D33" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="16.5">
+      <c r="A34" s="26"/>
+      <c r="B34" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="C34" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D34" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="16.5">
+      <c r="A35" s="26"/>
+      <c r="B35" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="C35" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D35" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="16.5">
+      <c r="A36" s="26"/>
+      <c r="B36" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="C36" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D36" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="16.5">
+      <c r="A37" s="26"/>
+      <c r="B37" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="C37" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D37" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B38" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="C38" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D38" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" s="26"/>
+      <c r="B39" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C39" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D39" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="26"/>
+      <c r="B40" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="C40" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D40" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="26"/>
+      <c r="B41" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C41" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D41" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" s="26"/>
+      <c r="B42" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="C42" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D42" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" s="26"/>
+      <c r="B43" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="C43" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D43" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" s="26"/>
+      <c r="B44" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="C44" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D44" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="16.5">
+      <c r="A45" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B45" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="C45" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D45" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" s="26"/>
+      <c r="B46" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C46" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D46" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="16.5">
+      <c r="A47" s="26"/>
+      <c r="B47" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="C47" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D47" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="16.5">
+      <c r="A48" s="26"/>
+      <c r="B48" s="24" t="s">
+        <v>45</v>
+      </c>
+      <c r="C48" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D48" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="16.5">
+      <c r="A49" s="26"/>
+      <c r="B49" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="C49" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D49" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="16.5">
+      <c r="A50" s="26"/>
+      <c r="B50" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C50" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D50" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="16.5">
+      <c r="A51" s="26"/>
+      <c r="B51" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C51" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D51" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="16.5">
+      <c r="A52" s="26"/>
+      <c r="B52" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="C52" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D52" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="16.5">
+      <c r="A53" s="26"/>
+      <c r="B53" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="C53" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D53" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="16.5">
+      <c r="A54" s="26"/>
+      <c r="B54" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="C54" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D54" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="16.5">
+      <c r="A55" s="26"/>
+      <c r="B55" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="C55" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D55" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="16.5">
+      <c r="A56" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="B56" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="C56" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D56" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="16.5">
+      <c r="A57" s="26"/>
+      <c r="B57" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="C57" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D57" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="16.5">
+      <c r="A58" s="26"/>
+      <c r="B58" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="C58" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D58" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="15" customHeight="1">
+      <c r="A59" s="26"/>
+      <c r="B59" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C59" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D59" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="15" customHeight="1">
+      <c r="A60" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="B60" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="C60" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D60" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="16.5">
+      <c r="A61" s="26"/>
+      <c r="B61" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="C61" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D61" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="15" customHeight="1">
+      <c r="A62" s="26"/>
+      <c r="B62" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="C62" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D62" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="16.5">
+      <c r="A63" s="26"/>
+      <c r="B63" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="C63" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D63" s="25" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" ht="15" customHeight="1">
+      <c r="A64" s="26"/>
+      <c r="B64" s="24" t="s">
+        <v>56</v>
+      </c>
+      <c r="C64" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D64" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="15" customHeight="1">
+      <c r="A65" s="26"/>
+      <c r="B65" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="C65" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D65" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="15" customHeight="1"/>
+    <row r="67" spans="1:4" ht="15" customHeight="1"/>
+    <row r="68" spans="1:4" ht="15" customHeight="1"/>
+    <row r="70" spans="1:4" ht="15" customHeight="1"/>
+    <row r="71" spans="1:4" ht="15" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F76D765B-9B47-4F6F-864D-2E742EEFE20A}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
@@ -701,38 +1775,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="12" t="s">
-        <v>0</v>
+      <c r="A1" s="13" t="s">
+        <v>58</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
+      <c r="C1" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="15"/>
-      <c r="B2" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:9" ht="23.25">
-      <c r="A3" s="15"/>
-      <c r="B3" s="13"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="16"/>
       <c r="C3" s="4" t="s">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="6"/>
@@ -742,10 +1816,10 @@
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:9" ht="23.25">
-      <c r="A4" s="15"/>
-      <c r="B4" s="13"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="4" t="s">
-        <v>4</v>
+        <v>62</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -755,12 +1829,12 @@
       <c r="I4" s="2"/>
     </row>
     <row r="5" spans="1:9" ht="23.25">
-      <c r="A5" s="15"/>
+      <c r="A5" s="14"/>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>6</v>
+        <v>64</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
@@ -770,12 +1844,12 @@
       <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:9" ht="23.25">
-      <c r="A6" s="15"/>
+      <c r="A6" s="14"/>
       <c r="B6" s="2" t="s">
-        <v>7</v>
+        <v>65</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -786,24 +1860,35 @@
     </row>
     <row r="7" spans="1:9" ht="18.75">
       <c r="A7" s="3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="10" t="s">
-        <v>12</v>
+        <v>67</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>68</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -813,18 +1898,19 @@
     <mergeCell ref="B2:B4"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8" xr:uid="{CEBAF748-5EE9-4100-85CE-A6FCD49B665A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8:B199" xr:uid="{CEBAF748-5EE9-4100-85CE-A6FCD49B665A}">
       <formula1>"Employee,SuperAdmin,HR Admin,Dean,IDC Admin,ISO Document Handler"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="A8" r:id="rId1" xr:uid="{394B655F-9F81-429C-A1EF-496E29AD8857}"/>
+    <hyperlink ref="A9" r:id="rId2" xr:uid="{5A76D44F-C0B2-4595-AD19-3EFF68E2DE8E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L50"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -844,16 +1930,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15" customHeight="1">
-      <c r="A1" s="12" t="s">
-        <v>0</v>
+      <c r="A1" s="13" t="s">
+        <v>58</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
+      <c r="C1" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
@@ -862,14 +1948,14 @@
       <c r="L1" s="2"/>
     </row>
     <row r="2" spans="1:12" ht="15" customHeight="1">
-      <c r="A2" s="12"/>
-      <c r="B2" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
@@ -878,10 +1964,10 @@
       <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:12" ht="23.25">
-      <c r="A3" s="12"/>
-      <c r="B3" s="13"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="16"/>
       <c r="C3" s="4" t="s">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="6"/>
@@ -894,10 +1980,10 @@
       <c r="L3" s="2"/>
     </row>
     <row r="4" spans="1:12" ht="23.25">
-      <c r="A4" s="12"/>
-      <c r="B4" s="13"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="4" t="s">
-        <v>4</v>
+        <v>62</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -910,12 +1996,12 @@
       <c r="L4" s="2"/>
     </row>
     <row r="5" spans="1:12" ht="23.25">
-      <c r="A5" s="12"/>
+      <c r="A5" s="13"/>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>6</v>
+        <v>64</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
@@ -928,12 +2014,12 @@
       <c r="L5" s="2"/>
     </row>
     <row r="6" spans="1:12" ht="23.25">
-      <c r="A6" s="12"/>
+      <c r="A6" s="13"/>
       <c r="B6" s="2" t="s">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -947,89 +2033,97 @@
     </row>
     <row r="7" spans="1:12" ht="18.75">
       <c r="A7" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8" s="8">
-        <v>54321</v>
+        <v>789745</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D8" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="12">
+        <v>36580</v>
+      </c>
+      <c r="I8" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="L8" s="8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" s="8">
+        <v>567899</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="G8" s="8" t="s">
+      <c r="C9" s="8"/>
+      <c r="D9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H8" s="9">
-        <v>37676</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="K8" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="L8" s="8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
+      <c r="E9" s="8" t="s">
+        <v>73</v>
+      </c>
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
+      <c r="H9" s="9"/>
       <c r="I9" s="8"/>
       <c r="J9" s="8"/>
       <c r="K9" s="8"/>
@@ -1631,7 +2725,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B5BD57D-7AE6-4F76-9833-54EA6E2059BD}">
   <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1650,38 +2744,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" customHeight="1">
-      <c r="A1" s="12" t="s">
-        <v>0</v>
+      <c r="A1" s="13" t="s">
+        <v>58</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
+      <c r="C1" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
     </row>
     <row r="2" spans="1:11" ht="15" customHeight="1">
-      <c r="A2" s="12"/>
-      <c r="B2" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:11" ht="23.25">
-      <c r="A3" s="12"/>
-      <c r="B3" s="13"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="16"/>
       <c r="C3" s="4" t="s">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="6"/>
@@ -1691,10 +2785,10 @@
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:11" ht="23.25">
-      <c r="A4" s="12"/>
-      <c r="B4" s="13"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="4" t="s">
-        <v>4</v>
+        <v>62</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -1704,12 +2798,12 @@
       <c r="I4" s="2"/>
     </row>
     <row r="5" spans="1:11" ht="23.25">
-      <c r="A5" s="12"/>
+      <c r="A5" s="13"/>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>6</v>
+        <v>64</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
@@ -1719,12 +2813,12 @@
       <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:11" ht="23.25">
-      <c r="A6" s="12"/>
+      <c r="A6" s="13"/>
       <c r="B6" s="2" t="s">
-        <v>32</v>
+        <v>77</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1735,34 +2829,34 @@
     </row>
     <row r="7" spans="1:11" ht="18.75">
       <c r="A7" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="H7" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="I7" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="J7" s="3" t="s">
         <v>41</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1770,16 +2864,16 @@
         <v>12345</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="D8" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="E8" s="8" t="s">
         <v>36</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>37</v>
       </c>
       <c r="F8" s="8">
         <v>2009</v>
@@ -1791,10 +2885,10 @@
         <v>987654321</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>12</v>
+        <v>67</v>
       </c>
       <c r="J8" s="11" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1879,7 +2973,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66B49A8D-A6EE-4466-9104-1F8E7FD48EC6}">
   <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1895,36 +2989,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="12" t="s">
-        <v>0</v>
+      <c r="A1" s="13" t="s">
+        <v>58</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
+      <c r="C1" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="15"/>
-      <c r="B2" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
     <row r="3" spans="1:8" ht="23.25">
-      <c r="A3" s="15"/>
-      <c r="B3" s="13"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="16"/>
       <c r="C3" s="4" t="s">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="6"/>
@@ -1933,10 +3027,10 @@
       <c r="H3" s="2"/>
     </row>
     <row r="4" spans="1:8" ht="23.25">
-      <c r="A4" s="15"/>
-      <c r="B4" s="13"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="4" t="s">
-        <v>4</v>
+        <v>62</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -1945,12 +3039,12 @@
       <c r="H4" s="2"/>
     </row>
     <row r="5" spans="1:8" ht="23.25">
-      <c r="A5" s="15"/>
+      <c r="A5" s="14"/>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>6</v>
+        <v>64</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
@@ -1959,12 +3053,12 @@
       <c r="H5" s="2"/>
     </row>
     <row r="6" spans="1:8" ht="23.25">
-      <c r="A6" s="15"/>
+      <c r="A6" s="14"/>
       <c r="B6" s="2" t="s">
-        <v>44</v>
+        <v>78</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -1974,25 +3068,25 @@
     </row>
     <row r="7" spans="1:8" ht="18.75">
       <c r="A7" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>38</v>
-      </c>
       <c r="G7" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -2000,16 +3094,16 @@
         <v>12345</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="D8" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="E8" s="8" t="s">
         <v>36</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>37</v>
       </c>
       <c r="F8" s="8">
         <v>2009</v>
@@ -2028,7 +3122,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{631417A2-3F94-413D-8C9F-DE5883DDF2FB}">
   <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2048,38 +3142,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="12" t="s">
-        <v>0</v>
+      <c r="A1" s="13" t="s">
+        <v>58</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
+      <c r="C1" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="15"/>
-      <c r="B2" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:11" ht="23.25">
-      <c r="A3" s="15"/>
-      <c r="B3" s="13"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="16"/>
       <c r="C3" s="4" t="s">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="6"/>
@@ -2089,10 +3183,10 @@
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:11" ht="23.25">
-      <c r="A4" s="15"/>
-      <c r="B4" s="13"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="4" t="s">
-        <v>4</v>
+        <v>62</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -2102,12 +3196,12 @@
       <c r="I4" s="2"/>
     </row>
     <row r="5" spans="1:11" ht="23.25">
-      <c r="A5" s="15"/>
+      <c r="A5" s="14"/>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>6</v>
+        <v>64</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
@@ -2117,12 +3211,12 @@
       <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:11" ht="23.25">
-      <c r="A6" s="15"/>
+      <c r="A6" s="14"/>
       <c r="B6" s="2" t="s">
-        <v>46</v>
+        <v>79</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -2133,63 +3227,63 @@
     </row>
     <row r="7" spans="1:11" ht="18.75">
       <c r="A7" s="3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E7" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>34</v>
-      </c>
       <c r="G7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="I7" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="J7" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="K7" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="8" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F8" s="8">
         <v>2009</v>
       </c>
       <c r="G8" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="H8" s="8" t="s">
         <v>36</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>37</v>
       </c>
       <c r="I8" s="8">
         <v>2009</v>
@@ -2211,7 +3305,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6938CC6A-1CF5-4A7A-B513-57A570803E03}">
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2223,38 +3317,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" customHeight="1">
-      <c r="A1" s="12" t="s">
-        <v>0</v>
+      <c r="A1" s="13" t="s">
+        <v>58</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
+      <c r="C1" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="12"/>
-      <c r="B2" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:9" ht="23.25">
-      <c r="A3" s="12"/>
-      <c r="B3" s="13"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="16"/>
       <c r="C3" s="4" t="s">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="6"/>
@@ -2264,10 +3358,10 @@
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:9" ht="23.25">
-      <c r="A4" s="12"/>
-      <c r="B4" s="13"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="4" t="s">
-        <v>4</v>
+        <v>62</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -2277,12 +3371,12 @@
       <c r="I4" s="2"/>
     </row>
     <row r="5" spans="1:9" ht="23.25">
-      <c r="A5" s="12"/>
+      <c r="A5" s="13"/>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>6</v>
+        <v>64</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
@@ -2292,12 +3386,12 @@
       <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:9" ht="23.25">
-      <c r="A6" s="12"/>
+      <c r="A6" s="13"/>
       <c r="B6" s="2" t="s">
-        <v>48</v>
+        <v>80</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -2308,16 +3402,16 @@
     </row>
     <row r="7" spans="1:9" ht="18.75">
       <c r="A7" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2344,7 +3438,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C52857AB-AEB0-4FAC-8863-55C98796A1A1}">
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2358,38 +3452,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="12" t="s">
-        <v>0</v>
+      <c r="A1" s="13" t="s">
+        <v>58</v>
       </c>
       <c r="B1" s="1"/>
-      <c r="C1" s="14" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
+      <c r="C1" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="15"/>
-      <c r="B2" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:9" ht="23.25">
-      <c r="A3" s="15"/>
-      <c r="B3" s="13"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="16"/>
       <c r="C3" s="4" t="s">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="6"/>
@@ -2399,10 +3493,10 @@
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:9" ht="23.25">
-      <c r="A4" s="15"/>
-      <c r="B4" s="13"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="4" t="s">
-        <v>4</v>
+        <v>62</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
@@ -2412,12 +3506,12 @@
       <c r="I4" s="2"/>
     </row>
     <row r="5" spans="1:9" ht="23.25">
-      <c r="A5" s="15"/>
+      <c r="A5" s="14"/>
       <c r="B5" s="2" t="s">
-        <v>5</v>
+        <v>63</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>6</v>
+        <v>64</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
@@ -2427,12 +3521,12 @@
       <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:9" ht="23.25">
-      <c r="A6" s="15"/>
+      <c r="A6" s="14"/>
       <c r="B6" s="2" t="s">
-        <v>53</v>
+        <v>83</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -2443,22 +3537,22 @@
     </row>
     <row r="7" spans="1:9" ht="18.75">
       <c r="A7" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>57</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2466,16 +3560,16 @@
         <v>44981</v>
       </c>
       <c r="B8" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="C8" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="D8" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="F8" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>